<commit_message>
add test for ApplyDefaultPermissions
</commit_message>
<xml_diff>
--- a/Scripts/Examples/Matrix template.xlsx
+++ b/Scripts/Examples/Matrix template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gijbelsb\Downloads\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE82312-BDE2-48AB-B5D4-9D3D52B8A813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6924A6DC-5608-43A7-BA57-D9067AEA4462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32250" yWindow="1785" windowWidth="21600" windowHeight="11235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Permissions" sheetId="4" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="54">
   <si>
     <t>F</t>
   </si>
@@ -289,6 +289,9 @@
   </si>
   <si>
     <t>COMPUTER2</t>
+  </si>
+  <si>
+    <t>ApplyDefaultPermissions</t>
   </si>
 </sst>
 </file>
@@ -2287,17 +2290,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" style="71" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" style="71" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -2313,11 +2317,14 @@
       <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="69" t="s">
+      <c r="F1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2333,11 +2340,14 @@
       <c r="E2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="70" t="s">
+      <c r="F2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="70" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
@@ -2353,105 +2363,120 @@
       <c r="E3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="70" t="s">
+      <c r="F3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="70" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D4" s="3"/>
       <c r="E4" s="4"/>
-      <c r="F4" s="70"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F4" s="4"/>
+      <c r="G4" s="70"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5" s="1"/>
       <c r="D5" s="3"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="70"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F5" s="4"/>
+      <c r="G5" s="70"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6" s="4"/>
       <c r="D6" s="3"/>
       <c r="E6" s="4"/>
-      <c r="F6" s="70"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F6" s="4"/>
+      <c r="G6" s="70"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="70"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7" s="4"/>
+      <c r="G7" s="70"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="70"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F8" s="4"/>
+      <c r="G8" s="70"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B9" s="4"/>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="70"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F9" s="4"/>
+      <c r="G9" s="70"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B10" s="1"/>
       <c r="D10" s="3"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="70"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="4"/>
+      <c r="G10" s="70"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D11" s="3"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="70"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F11" s="4"/>
+      <c r="G11" s="70"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B12" s="1"/>
       <c r="D12" s="3"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="70"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F12" s="4"/>
+      <c r="G12" s="70"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B13" s="4"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="70"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F13" s="4"/>
+      <c r="G13" s="70"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B14" s="4"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="70"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F14" s="4"/>
+      <c r="G14" s="70"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B15" s="4"/>
       <c r="D15" s="3"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="70"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F15" s="4"/>
+      <c r="G15" s="70"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B16" s="4"/>
-      <c r="F16" s="70"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="G16" s="70"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="4"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
-      <c r="F17" s="70"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="G17" s="70"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="4"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
-      <c r="F18" s="70"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="G18" s="70"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="4"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-      <c r="F19" s="70"/>
+      <c r="G19" s="70"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2703,9 +2728,7 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2758,7 +2781,9 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2771,16 +2796,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AE7EF8E-BF67-4561-A935-3685C3E9EC35}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAB8DE14-8EA8-40DE-9709-400EEAA9E777}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2801,9 +2819,16 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAB8DE14-8EA8-40DE-9709-400EEAA9E777}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AE7EF8E-BF67-4561-A935-3685C3E9EC35}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>